<commit_message>
fixes to file names
</commit_message>
<xml_diff>
--- a/fields.xlsx
+++ b/fields.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jonny\Dev\Osu-Skin-Helper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC5897C9-AB0C-4690-8119-9A645B2956A8}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DD77838-CAF7-4064-A14F-49170A04529E}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{C5EE6F83-43A7-42CD-8E46-C6413A8819FF}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="861" uniqueCount="315">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="861" uniqueCount="317">
   <si>
     <t>sprite-name(@2x).png</t>
   </si>
@@ -979,6 +979,12 @@
   </si>
   <si>
     <t>score_numbers</t>
+  </si>
+  <si>
+    <t>hitcircle_object</t>
+  </si>
+  <si>
+    <t>taiko_drumroll</t>
   </si>
 </sst>
 </file>
@@ -1340,6 +1346,7 @@
   <dimension ref="A1:C287"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="2" max="2" width="21" customWidth="1"/>
     <col min="3" max="3" width="113.85546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3152,7 +3159,7 @@
         <v>282</v>
       </c>
       <c r="B165" t="s">
-        <v>297</v>
+        <v>315</v>
       </c>
       <c r="C165" t="s">
         <v>162</v>
@@ -3163,7 +3170,7 @@
         <v>282</v>
       </c>
       <c r="B166" t="s">
-        <v>297</v>
+        <v>315</v>
       </c>
       <c r="C166" t="s">
         <v>163</v>
@@ -3174,7 +3181,7 @@
         <v>282</v>
       </c>
       <c r="B167" t="s">
-        <v>297</v>
+        <v>315</v>
       </c>
       <c r="C167" t="s">
         <v>164</v>
@@ -3185,7 +3192,7 @@
         <v>282</v>
       </c>
       <c r="B168" t="s">
-        <v>297</v>
+        <v>315</v>
       </c>
       <c r="C168" t="s">
         <v>165</v>
@@ -3196,7 +3203,7 @@
         <v>282</v>
       </c>
       <c r="B169" t="s">
-        <v>297</v>
+        <v>315</v>
       </c>
       <c r="C169" t="s">
         <v>166</v>
@@ -3207,7 +3214,7 @@
         <v>282</v>
       </c>
       <c r="B170" t="s">
-        <v>297</v>
+        <v>315</v>
       </c>
       <c r="C170" t="s">
         <v>167</v>
@@ -3218,7 +3225,7 @@
         <v>282</v>
       </c>
       <c r="B171" t="s">
-        <v>297</v>
+        <v>315</v>
       </c>
       <c r="C171" t="s">
         <v>168</v>
@@ -3229,7 +3236,7 @@
         <v>282</v>
       </c>
       <c r="B172" t="s">
-        <v>297</v>
+        <v>315</v>
       </c>
       <c r="C172" t="s">
         <v>169</v>
@@ -3240,7 +3247,7 @@
         <v>282</v>
       </c>
       <c r="B173" t="s">
-        <v>297</v>
+        <v>315</v>
       </c>
       <c r="C173" t="s">
         <v>170</v>
@@ -3812,7 +3819,7 @@
         <v>283</v>
       </c>
       <c r="B225" t="s">
-        <v>304</v>
+        <v>316</v>
       </c>
       <c r="C225" t="s">
         <v>220</v>
@@ -3823,7 +3830,7 @@
         <v>283</v>
       </c>
       <c r="B226" t="s">
-        <v>304</v>
+        <v>316</v>
       </c>
       <c r="C226" t="s">
         <v>221</v>
@@ -3834,7 +3841,7 @@
         <v>283</v>
       </c>
       <c r="B227" t="s">
-        <v>304</v>
+        <v>316</v>
       </c>
       <c r="C227" t="s">
         <v>175</v>
@@ -3845,7 +3852,7 @@
         <v>283</v>
       </c>
       <c r="B228" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C228" t="s">
         <v>222</v>
@@ -3856,7 +3863,7 @@
         <v>283</v>
       </c>
       <c r="B229" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C229" t="s">
         <v>177</v>
@@ -3867,7 +3874,7 @@
         <v>283</v>
       </c>
       <c r="B230" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C230" t="s">
         <v>184</v>

</xml_diff>